<commit_message>
feat(prototipo): Idealista también lee la tabla de los últimos 12 meses de España
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/prototipos/carga_manual/idealista_prototipo.xlsx
+++ b/prototipos/carga_manual/idealista_prototipo.xlsx
@@ -16,7 +16,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Tablas'!$A$1:$K$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Campos'!$A$1:$H$49</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'idealista_precio_alquiler'!$A$2:$X$29</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'idealista_precio_venta'!$A$2:$X$31</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'idealista_precio_venta'!$A$2:$X$42</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -670,7 +670,7 @@
         </is>
       </c>
       <c r="J3" s="2" t="n">
-        <v>29</v>
+        <v>40</v>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
@@ -4692,7 +4692,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X31"/>
+  <dimension ref="A1:X42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4724,7 +4724,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>Muestra: 29 de 29 filas. La tabla completa está en prototipos/carga_manual/salida/idealista_precio_venta.csv</t>
+          <t>Muestra: 40 de 40 filas. La tabla completa está en prototipos/carga_manual/salida/idealista_precio_venta.csv</t>
         </is>
       </c>
     </row>
@@ -7115,8 +7115,712 @@
         <v>46325</v>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" s="7" t="inlineStr">
+        <is>
+          <t>ES_2026M08</t>
+        </is>
+      </c>
+      <c r="B32" s="7" t="inlineStr">
+        <is>
+          <t>Nacional</t>
+        </is>
+      </c>
+      <c r="C32" s="8" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D32" s="8" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="E32" s="7" t="inlineStr">
+        <is>
+          <t>Total Nacional</t>
+        </is>
+      </c>
+      <c r="J32" s="7" t="inlineStr">
+        <is>
+          <t>2026M08</t>
+        </is>
+      </c>
+      <c r="K32" s="7" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="L32" s="7" t="n">
+        <v>2026</v>
+      </c>
+      <c r="N32" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="O32" s="9" t="n">
+        <v>46235</v>
+      </c>
+      <c r="P32" s="7" t="n">
+        <v>2924</v>
+      </c>
+      <c r="Q32" s="7" t="n">
+        <v>-0.3</v>
+      </c>
+      <c r="R32" s="7" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="S32" s="7" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="W32" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="X32" s="9" t="n">
+        <v>46325</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="7" t="inlineStr">
+        <is>
+          <t>ES_2026M07</t>
+        </is>
+      </c>
+      <c r="B33" s="7" t="inlineStr">
+        <is>
+          <t>Nacional</t>
+        </is>
+      </c>
+      <c r="C33" s="8" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D33" s="8" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="E33" s="7" t="inlineStr">
+        <is>
+          <t>Total Nacional</t>
+        </is>
+      </c>
+      <c r="J33" s="7" t="inlineStr">
+        <is>
+          <t>2026M07</t>
+        </is>
+      </c>
+      <c r="K33" s="7" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="L33" s="7" t="n">
+        <v>2026</v>
+      </c>
+      <c r="N33" s="7" t="n">
+        <v>7</v>
+      </c>
+      <c r="O33" s="9" t="n">
+        <v>46204</v>
+      </c>
+      <c r="P33" s="7" t="n">
+        <v>2933</v>
+      </c>
+      <c r="Q33" s="7" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="R33" s="7" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="S33" s="7" t="n">
+        <v>13.1</v>
+      </c>
+      <c r="W33" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="X33" s="9" t="n">
+        <v>46325</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="7" t="inlineStr">
+        <is>
+          <t>ES_2026M06</t>
+        </is>
+      </c>
+      <c r="B34" s="7" t="inlineStr">
+        <is>
+          <t>Nacional</t>
+        </is>
+      </c>
+      <c r="C34" s="8" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D34" s="8" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="E34" s="7" t="inlineStr">
+        <is>
+          <t>Total Nacional</t>
+        </is>
+      </c>
+      <c r="J34" s="7" t="inlineStr">
+        <is>
+          <t>2026M06</t>
+        </is>
+      </c>
+      <c r="K34" s="7" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="L34" s="7" t="n">
+        <v>2026</v>
+      </c>
+      <c r="N34" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="O34" s="9" t="n">
+        <v>46174</v>
+      </c>
+      <c r="P34" s="7" t="n">
+        <v>2914</v>
+      </c>
+      <c r="Q34" s="7" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="R34" s="7" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="S34" s="7" t="n">
+        <v>13.9</v>
+      </c>
+      <c r="W34" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="X34" s="9" t="n">
+        <v>46325</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="7" t="inlineStr">
+        <is>
+          <t>ES_2026M05</t>
+        </is>
+      </c>
+      <c r="B35" s="7" t="inlineStr">
+        <is>
+          <t>Nacional</t>
+        </is>
+      </c>
+      <c r="C35" s="8" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D35" s="8" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="E35" s="7" t="inlineStr">
+        <is>
+          <t>Total Nacional</t>
+        </is>
+      </c>
+      <c r="J35" s="7" t="inlineStr">
+        <is>
+          <t>2026M05</t>
+        </is>
+      </c>
+      <c r="K35" s="7" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="L35" s="7" t="n">
+        <v>2026</v>
+      </c>
+      <c r="N35" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="O35" s="9" t="n">
+        <v>46143</v>
+      </c>
+      <c r="P35" s="7" t="n">
+        <v>2881</v>
+      </c>
+      <c r="Q35" s="7" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="R35" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="S35" s="7" t="n">
+        <v>14.7</v>
+      </c>
+      <c r="W35" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="X35" s="9" t="n">
+        <v>46325</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="7" t="inlineStr">
+        <is>
+          <t>ES_2026M04</t>
+        </is>
+      </c>
+      <c r="B36" s="7" t="inlineStr">
+        <is>
+          <t>Nacional</t>
+        </is>
+      </c>
+      <c r="C36" s="8" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D36" s="8" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="E36" s="7" t="inlineStr">
+        <is>
+          <t>Total Nacional</t>
+        </is>
+      </c>
+      <c r="J36" s="7" t="inlineStr">
+        <is>
+          <t>2026M04</t>
+        </is>
+      </c>
+      <c r="K36" s="7" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="L36" s="7" t="n">
+        <v>2026</v>
+      </c>
+      <c r="N36" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="O36" s="9" t="n">
+        <v>46113</v>
+      </c>
+      <c r="P36" s="7" t="n">
+        <v>2839</v>
+      </c>
+      <c r="Q36" s="7" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="R36" s="7" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="S36" s="7" t="n">
+        <v>15</v>
+      </c>
+      <c r="W36" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="X36" s="9" t="n">
+        <v>46325</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="7" t="inlineStr">
+        <is>
+          <t>ES_2026M03</t>
+        </is>
+      </c>
+      <c r="B37" s="7" t="inlineStr">
+        <is>
+          <t>Nacional</t>
+        </is>
+      </c>
+      <c r="C37" s="8" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D37" s="8" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="E37" s="7" t="inlineStr">
+        <is>
+          <t>Total Nacional</t>
+        </is>
+      </c>
+      <c r="J37" s="7" t="inlineStr">
+        <is>
+          <t>2026M03</t>
+        </is>
+      </c>
+      <c r="K37" s="7" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="L37" s="7" t="n">
+        <v>2026</v>
+      </c>
+      <c r="N37" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="O37" s="9" t="n">
+        <v>46082</v>
+      </c>
+      <c r="P37" s="7" t="n">
+        <v>2807</v>
+      </c>
+      <c r="Q37" s="7" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="R37" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="S37" s="7" t="n">
+        <v>16</v>
+      </c>
+      <c r="W37" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="X37" s="9" t="n">
+        <v>46325</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="7" t="inlineStr">
+        <is>
+          <t>ES_2026M02</t>
+        </is>
+      </c>
+      <c r="B38" s="7" t="inlineStr">
+        <is>
+          <t>Nacional</t>
+        </is>
+      </c>
+      <c r="C38" s="8" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D38" s="8" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="E38" s="7" t="inlineStr">
+        <is>
+          <t>Total Nacional</t>
+        </is>
+      </c>
+      <c r="J38" s="7" t="inlineStr">
+        <is>
+          <t>2026M02</t>
+        </is>
+      </c>
+      <c r="K38" s="7" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="L38" s="7" t="n">
+        <v>2026</v>
+      </c>
+      <c r="N38" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="O38" s="9" t="n">
+        <v>46054</v>
+      </c>
+      <c r="P38" s="7" t="n">
+        <v>2771</v>
+      </c>
+      <c r="Q38" s="7" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="R38" s="7" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="S38" s="7" t="n">
+        <v>16.4</v>
+      </c>
+      <c r="W38" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="X38" s="9" t="n">
+        <v>46325</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="7" t="inlineStr">
+        <is>
+          <t>ES_2026M01</t>
+        </is>
+      </c>
+      <c r="B39" s="7" t="inlineStr">
+        <is>
+          <t>Nacional</t>
+        </is>
+      </c>
+      <c r="C39" s="8" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D39" s="8" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="E39" s="7" t="inlineStr">
+        <is>
+          <t>Total Nacional</t>
+        </is>
+      </c>
+      <c r="J39" s="7" t="inlineStr">
+        <is>
+          <t>2026M01</t>
+        </is>
+      </c>
+      <c r="K39" s="7" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="L39" s="7" t="n">
+        <v>2026</v>
+      </c>
+      <c r="N39" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="O39" s="9" t="n">
+        <v>46023</v>
+      </c>
+      <c r="P39" s="7" t="n">
+        <v>2739</v>
+      </c>
+      <c r="Q39" s="7" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="R39" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="S39" s="7" t="n">
+        <v>16.8</v>
+      </c>
+      <c r="W39" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="X39" s="9" t="n">
+        <v>46325</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="7" t="inlineStr">
+        <is>
+          <t>ES_2025M12</t>
+        </is>
+      </c>
+      <c r="B40" s="7" t="inlineStr">
+        <is>
+          <t>Nacional</t>
+        </is>
+      </c>
+      <c r="C40" s="8" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D40" s="8" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="E40" s="7" t="inlineStr">
+        <is>
+          <t>Total Nacional</t>
+        </is>
+      </c>
+      <c r="J40" s="7" t="inlineStr">
+        <is>
+          <t>2025M12</t>
+        </is>
+      </c>
+      <c r="K40" s="7" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="L40" s="7" t="n">
+        <v>2025</v>
+      </c>
+      <c r="N40" s="7" t="n">
+        <v>12</v>
+      </c>
+      <c r="O40" s="9" t="n">
+        <v>45992</v>
+      </c>
+      <c r="P40" s="7" t="n">
+        <v>2725</v>
+      </c>
+      <c r="Q40" s="7" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R40" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="S40" s="7" t="n">
+        <v>17.2</v>
+      </c>
+      <c r="W40" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="X40" s="9" t="n">
+        <v>46325</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="7" t="inlineStr">
+        <is>
+          <t>ES_2025M11</t>
+        </is>
+      </c>
+      <c r="B41" s="7" t="inlineStr">
+        <is>
+          <t>Nacional</t>
+        </is>
+      </c>
+      <c r="C41" s="8" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D41" s="8" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="E41" s="7" t="inlineStr">
+        <is>
+          <t>Total Nacional</t>
+        </is>
+      </c>
+      <c r="J41" s="7" t="inlineStr">
+        <is>
+          <t>2025M11</t>
+        </is>
+      </c>
+      <c r="K41" s="7" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="L41" s="7" t="n">
+        <v>2025</v>
+      </c>
+      <c r="N41" s="7" t="n">
+        <v>11</v>
+      </c>
+      <c r="O41" s="9" t="n">
+        <v>45962</v>
+      </c>
+      <c r="P41" s="7" t="n">
+        <v>2701</v>
+      </c>
+      <c r="Q41" s="7" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="R41" s="7" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="S41" s="7" t="n">
+        <v>16.8</v>
+      </c>
+      <c r="W41" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="X41" s="9" t="n">
+        <v>46325</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="7" t="inlineStr">
+        <is>
+          <t>ES_2025M10</t>
+        </is>
+      </c>
+      <c r="B42" s="7" t="inlineStr">
+        <is>
+          <t>Nacional</t>
+        </is>
+      </c>
+      <c r="C42" s="8" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D42" s="8" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="E42" s="7" t="inlineStr">
+        <is>
+          <t>Total Nacional</t>
+        </is>
+      </c>
+      <c r="J42" s="7" t="inlineStr">
+        <is>
+          <t>2025M10</t>
+        </is>
+      </c>
+      <c r="K42" s="7" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="L42" s="7" t="n">
+        <v>2025</v>
+      </c>
+      <c r="N42" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="O42" s="9" t="n">
+        <v>45931</v>
+      </c>
+      <c r="P42" s="7" t="n">
+        <v>2658</v>
+      </c>
+      <c r="Q42" s="7" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="R42" s="7" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="S42" s="7" t="n">
+        <v>16.6</v>
+      </c>
+      <c r="W42" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="X42" s="9" t="n">
+        <v>46325</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:X31"/>
+  <autoFilter ref="A2:X42"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>